<commit_message>
Complete le lot 2 a 35 prospects
Ajoute 1 artisan et 2 services de proximite, le vivier ayant grossi
depuis le scan complementaire.

Ecarte deux faux prospects reperes a la main : gad.touchnpay.fr est la
plateforme de paiement d'une laverie et lille.demosphere.net un agenda
associatif - dans les deux cas le pro n'a pas la main sur le site.
Leurs domaines rejoignent la liste des plateformes.

Corrige deux noms depuis les sites eux-memes : OSM donnait
'Ambert icorni' pour Lambert Licorni, et le nom du gerant au lieu de
l'enseigne pour CS2M.
</commit_message>
<xml_diff>
--- a/lot_02.xlsx
+++ b/lot_02.xlsx
@@ -14,11 +14,11 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Services de proximite" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Artisanat &amp; BTP'!$A$3:$J$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Artisanat &amp; BTP'!$A$3:$J$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Beaute &amp; Bien-etre'!$A$3:$J$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Restauration'!$A$3:$J$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Automobile'!$A$3:$J$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Services de proximite'!$A$3:$J$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Services de proximite'!$A$3:$J$10</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -67,7 +67,7 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0092400E"/>
+      <color rgb="00991B1B"/>
       <sz val="11"/>
     </font>
     <font>
@@ -89,13 +89,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00374151"/>
+      <color rgb="0092400E"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00991B1B"/>
+      <color rgb="00374151"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -113,7 +113,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEF3C7"/>
+        <fgColor rgb="00FEE2E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -123,12 +123,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F3F4F6"/>
+        <fgColor rgb="00FEF3C7"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEE2E2"/>
+        <fgColor rgb="00F3F4F6"/>
       </patternFill>
     </fill>
   </fills>
@@ -206,7 +206,13 @@
     <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -214,12 +220,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -589,7 +589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -607,7 +607,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Artisanat &amp; BTP  ·  6 prospects</t>
+          <t>Artisanat &amp; BTP  ·  7 prospects</t>
         </is>
       </c>
     </row>
@@ -673,29 +673,29 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>celo-gaz.com</t>
+          <t>lambert-licorni.fr</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Celo gaz</t>
+          <t>Lambert Licorni</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Nancy</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>75</t>
+          <t>54</t>
         </is>
       </c>
       <c r="E4" s="8" t="n">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
@@ -714,93 +714,93 @@
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
+          <t>balises &lt;font&gt; (16) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>atelier-delaunay.fr</t>
+          <t>celo-gaz.com</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>Atelier Delaunay</t>
+          <t>Celo gaz</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Le Havre</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>76</t>
-        </is>
-      </c>
-      <c r="E5" s="8" t="n">
-        <v>41</v>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E5" s="17" t="n">
+        <v>46</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="G5" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H5" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J5" s="19" t="inlineStr">
-        <is>
-          <t>layout en tableaux (25) | bgcolor= | doctype ancien | non responsive | &lt;br&gt; en masse</t>
+        <v>3</v>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>h4b.fr</t>
+          <t>atelier-delaunay.fr</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Henri De Quatres Barbes</t>
+          <t>Atelier Delaunay</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Le Havre</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="E6" s="8" t="n">
-        <v>39</v>
+          <t>76</t>
+        </is>
+      </c>
+      <c r="E6" s="17" t="n">
+        <v>41</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G6" s="9" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>oui</t>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -810,19 +810,19 @@
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>doctype ancien | non responsive | images .gif | pas de @media | pas de variables CSS</t>
+          <t>layout en tableaux (25) | bgcolor= | doctype ancien | non responsive | &lt;br&gt; en masse</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>begrand.fr</t>
+          <t>h4b.fr</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Entreprise Begrand</t>
+          <t>Henri De Quatres Barbes</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
@@ -835,68 +835,68 @@
           <t>75</t>
         </is>
       </c>
-      <c r="E7" s="20" t="n">
-        <v>33</v>
+      <c r="E7" s="17" t="n">
+        <v>39</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="G7" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H7" s="21" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J7" s="19" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (3) | doctype ancien | non responsive | document.write</t>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J7" s="21" t="inlineStr">
+        <is>
+          <t>doctype ancien | non responsive | images .gif | pas de @media | pas de variables CSS</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>brunelli.fr</t>
+          <t>begrand.fr</t>
         </is>
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Brunelli</t>
+          <t>Entreprise Begrand</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Nancy</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
-          <t>54</t>
-        </is>
-      </c>
-      <c r="E8" s="20" t="n">
-        <v>29</v>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="n">
+        <v>33</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G8" s="9" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="H8" s="9" t="inlineStr">
-        <is>
-          <t>non</t>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>oui</t>
         </is>
       </c>
       <c r="I8" s="11" t="inlineStr">
@@ -906,60 +906,108 @@
       </c>
       <c r="J8" s="12" t="inlineStr">
         <is>
-          <t>frameset | doctype ancien | non responsive</t>
+          <t>balises &lt;font&gt; (3) | doctype ancien | non responsive | document.write</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="13" t="inlineStr">
         <is>
+          <t>brunelli.fr</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Brunelli</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Nancy</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>29</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J9" s="21" t="inlineStr">
+        <is>
+          <t>frameset | doctype ancien | non responsive</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>alazard-sas.com</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>Alazard</t>
         </is>
       </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D9" s="16" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E10" s="22" t="n">
         <v>29</v>
       </c>
-      <c r="F9" s="16" t="n">
+      <c r="F10" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H9" s="21" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I9" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J9" s="19" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>non responsive | pas de @media</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J9"/>
+  <autoFilter ref="A3:J10"/>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
@@ -971,6 +1019,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId5"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1084,7 +1133,7 @@
           <t>44</t>
         </is>
       </c>
-      <c r="E4" s="22" t="n">
+      <c r="E4" s="8" t="n">
         <v>56</v>
       </c>
       <c r="F4" s="7" t="n">
@@ -1132,28 +1181,28 @@
           <t>69</t>
         </is>
       </c>
-      <c r="E5" s="22" t="n">
+      <c r="E5" s="8" t="n">
         <v>56</v>
       </c>
       <c r="F5" s="16" t="n">
         <v>6</v>
       </c>
-      <c r="G5" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H5" s="21" t="inlineStr">
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J5" s="19" t="inlineStr">
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>balises &lt;font&gt; (48) | non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
@@ -1180,7 +1229,7 @@
           <t>75</t>
         </is>
       </c>
-      <c r="E6" s="22" t="n">
+      <c r="E6" s="8" t="n">
         <v>56</v>
       </c>
       <c r="F6" s="7" t="n">
@@ -1228,28 +1277,28 @@
           <t>69</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="17" t="n">
         <v>46</v>
       </c>
       <c r="F7" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H7" s="21" t="inlineStr">
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J7" s="19" t="inlineStr">
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | CSS tres court (434B) | aucun radius/ombre</t>
         </is>
@@ -1276,7 +1325,7 @@
           <t>75</t>
         </is>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="17" t="n">
         <v>46</v>
       </c>
       <c r="F8" s="7" t="n">
@@ -1324,28 +1373,28 @@
           <t>76</t>
         </is>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="17" t="n">
         <v>42</v>
       </c>
       <c r="F9" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H9" s="21" t="inlineStr">
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H9" s="19" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I9" s="18" t="inlineStr">
+      <c r="I9" s="20" t="inlineStr">
         <is>
           <t>webacappella 4.6.18 free (win)</t>
         </is>
       </c>
-      <c r="J9" s="19" t="inlineStr">
+      <c r="J9" s="21" t="inlineStr">
         <is>
           <t>doctype ancien | non responsive | document.write | pas de @media | pas de flex/grid</t>
         </is>
@@ -1372,7 +1421,7 @@
           <t>75</t>
         </is>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="17" t="n">
         <v>41</v>
       </c>
       <c r="F10" s="7" t="n">
@@ -1526,7 +1575,7 @@
           <t>31</t>
         </is>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="17" t="n">
         <v>42</v>
       </c>
       <c r="F4" s="7" t="n">
@@ -1574,28 +1623,28 @@
           <t>75</t>
         </is>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="17" t="n">
         <v>39</v>
       </c>
       <c r="F5" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="G5" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H5" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J5" s="19" t="inlineStr">
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>layout en tableaux (8) | bgcolor= | sans doctype | non responsive</t>
         </is>
@@ -1622,7 +1671,7 @@
           <t>31</t>
         </is>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="17" t="n">
         <v>39</v>
       </c>
       <c r="F6" s="7" t="n">
@@ -1670,28 +1719,28 @@
           <t>31</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="17" t="n">
         <v>38</v>
       </c>
       <c r="F7" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="G7" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H7" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H7" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
         <is>
           <t>wordpress 3.7.41</t>
         </is>
       </c>
-      <c r="J7" s="19" t="inlineStr">
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>doctype ancien | non responsive | pas de @media | pas de flex/grid</t>
         </is>
@@ -1718,7 +1767,7 @@
           <t>69</t>
         </is>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="17" t="n">
         <v>37</v>
       </c>
       <c r="F8" s="7" t="n">
@@ -1766,28 +1815,28 @@
           <t>75</t>
         </is>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="17" t="n">
         <v>37</v>
       </c>
       <c r="F9" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H9" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I9" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J9" s="19" t="inlineStr">
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J9" s="21" t="inlineStr">
         <is>
           <t>non responsive | document.write | pas de @media | police vintage</t>
         </is>
@@ -1814,7 +1863,7 @@
           <t>59</t>
         </is>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="17" t="n">
         <v>37</v>
       </c>
       <c r="F10" s="7" t="n">
@@ -1968,7 +2017,7 @@
           <t>49</t>
         </is>
       </c>
-      <c r="E4" s="8" t="n">
+      <c r="E4" s="17" t="n">
         <v>46</v>
       </c>
       <c r="F4" s="7" t="n">
@@ -2016,28 +2065,28 @@
           <t>69</t>
         </is>
       </c>
-      <c r="E5" s="8" t="n">
+      <c r="E5" s="17" t="n">
         <v>44</v>
       </c>
       <c r="F5" s="16" t="n">
         <v>5</v>
       </c>
-      <c r="G5" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H5" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I5" s="18" t="inlineStr">
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H5" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I5" s="20" t="inlineStr">
         <is>
           <t>spip 3.1.3 [23214] - sarka-spip 3.4.6 [99617]</t>
         </is>
       </c>
-      <c r="J5" s="19" t="inlineStr">
+      <c r="J5" s="21" t="inlineStr">
         <is>
           <t>non responsive | images .gif | document.write | pas de @media | pas de flex/grid | aucun radius/ombre</t>
         </is>
@@ -2064,7 +2113,7 @@
           <t>35</t>
         </is>
       </c>
-      <c r="E6" s="8" t="n">
+      <c r="E6" s="17" t="n">
         <v>41</v>
       </c>
       <c r="F6" s="7" t="n">
@@ -2112,28 +2161,28 @@
           <t>57</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="17" t="n">
         <v>41</v>
       </c>
       <c r="F7" s="16" t="n">
         <v>3</v>
       </c>
-      <c r="G7" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H7" s="21" t="inlineStr">
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J7" s="19" t="inlineStr">
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>non responsive | pas de @media | pas de flex/grid | pas de variables CSS | police vintage</t>
         </is>
@@ -2160,7 +2209,7 @@
           <t>44</t>
         </is>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="22" t="n">
         <v>32</v>
       </c>
       <c r="F8" s="7" t="n">
@@ -2208,28 +2257,28 @@
           <t>25</t>
         </is>
       </c>
-      <c r="E9" s="20" t="n">
+      <c r="E9" s="22" t="n">
         <v>29</v>
       </c>
       <c r="F9" s="16" t="n">
         <v>8</v>
       </c>
-      <c r="G9" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H9" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I9" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J9" s="19" t="inlineStr">
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J9" s="21" t="inlineStr">
         <is>
           <t>frameset | doctype ancien | non responsive</t>
         </is>
@@ -2256,7 +2305,7 @@
           <t>30</t>
         </is>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="22" t="n">
         <v>25</v>
       </c>
       <c r="F10" s="7" t="n">
@@ -2308,7 +2357,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2326,7 +2375,7 @@
     <row r="1" ht="34" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Services de proximite  ·  5 prospects</t>
+          <t>Services de proximite  ·  7 prospects</t>
         </is>
       </c>
     </row>
@@ -2392,12 +2441,12 @@
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>pressingleluxembourg.com</t>
+          <t>depuy.free.fr</t>
         </is>
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>Le Luxembourg</t>
+          <t>SAV Depuy</t>
         </is>
       </c>
       <c r="C4" s="6" t="inlineStr">
@@ -2410,11 +2459,11 @@
           <t>75</t>
         </is>
       </c>
-      <c r="E4" s="20" t="n">
-        <v>32</v>
+      <c r="E4" s="17" t="n">
+        <v>38</v>
       </c>
       <c r="F4" s="7" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G4" s="9" t="inlineStr">
         <is>
@@ -2433,93 +2482,93 @@
       </c>
       <c r="J4" s="12" t="inlineStr">
         <is>
-          <t>non responsive | pas de @media | pas de variables CSS</t>
+          <t>balises &lt;font&gt; (57) | bgcolor= | sans doctype | non responsive | images .gif</t>
         </is>
       </c>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="13" t="inlineStr">
         <is>
-          <t>autourducycle.fr</t>
+          <t>cs2m.fr</t>
         </is>
       </c>
       <c r="B5" s="14" t="inlineStr">
         <is>
-          <t>Autour du Cycle</t>
+          <t>CS2M - Cordonnerie Serrurerie</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D5" s="16" t="inlineStr">
         <is>
-          <t>75</t>
-        </is>
-      </c>
-      <c r="E5" s="20" t="n">
-        <v>29</v>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="E5" s="22" t="n">
+        <v>34</v>
       </c>
       <c r="F5" s="16" t="n">
-        <v>6</v>
-      </c>
-      <c r="G5" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H5" s="21" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="G5" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H5" s="19" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I5" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J5" s="19" t="inlineStr">
-        <is>
-          <t>balises &lt;font&gt; (11) | non responsive | police vintage</t>
+      <c r="I5" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J5" s="21" t="inlineStr">
+        <is>
+          <t>non responsive | pas de @media | pas de flex/grid</t>
         </is>
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>alizes-pressing.fr</t>
+          <t>pressingleluxembourg.com</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t>Alizée Naturellement Pressing</t>
+          <t>Le Luxembourg</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>59</t>
-        </is>
-      </c>
-      <c r="E6" s="20" t="n">
-        <v>28</v>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E6" s="22" t="n">
+        <v>32</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="10" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>oui</t>
+        <v>5</v>
+      </c>
+      <c r="G6" s="9" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H6" s="9" t="inlineStr">
+        <is>
+          <t>non</t>
         </is>
       </c>
       <c r="I6" s="11" t="inlineStr">
@@ -2529,19 +2578,19 @@
       </c>
       <c r="J6" s="12" t="inlineStr">
         <is>
-          <t>pas de @media | pas de flex/grid | CSS tres court (506B) | aucun radius/ombre</t>
+          <t>non responsive | pas de @media | pas de variables CSS</t>
         </is>
       </c>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="13" t="inlineStr">
         <is>
-          <t>cycle-naturel.com</t>
+          <t>autourducycle.fr</t>
         </is>
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>Cycle Naturel</t>
+          <t>Autour du Cycle</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
@@ -2554,83 +2603,179 @@
           <t>75</t>
         </is>
       </c>
-      <c r="E7" s="20" t="n">
-        <v>25</v>
+      <c r="E7" s="22" t="n">
+        <v>29</v>
       </c>
       <c r="F7" s="16" t="n">
-        <v>8</v>
-      </c>
-      <c r="G7" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H7" s="17" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="I7" s="18" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J7" s="19" t="inlineStr">
-        <is>
-          <t>frameset | non responsive</t>
+        <v>6</v>
+      </c>
+      <c r="G7" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I7" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J7" s="21" t="inlineStr">
+        <is>
+          <t>balises &lt;font&gt; (11) | non responsive | police vintage</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
+          <t>alizes-pressing.fr</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>Alizée Naturellement Pressing</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Lille</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>59</t>
+        </is>
+      </c>
+      <c r="E8" s="22" t="n">
+        <v>28</v>
+      </c>
+      <c r="F8" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="10" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="I8" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J8" s="12" t="inlineStr">
+        <is>
+          <t>pas de @media | pas de flex/grid | CSS tres court (506B) | aucun radius/ombre</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>cycle-naturel.com</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr">
+        <is>
+          <t>Cycle Naturel</t>
+        </is>
+      </c>
+      <c r="C9" s="15" t="inlineStr">
+        <is>
+          <t>Paris</t>
+        </is>
+      </c>
+      <c r="D9" s="16" t="inlineStr">
+        <is>
+          <t>75</t>
+        </is>
+      </c>
+      <c r="E9" s="22" t="n">
+        <v>25</v>
+      </c>
+      <c r="F9" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G9" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H9" s="18" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="I9" s="20" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J9" s="21" t="inlineStr">
+        <is>
+          <t>frameset | non responsive</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
           <t>3dinfomac.com</t>
         </is>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B10" s="5" t="inlineStr">
         <is>
           <t>3D Informatique</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Paris</t>
         </is>
       </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="D10" s="7" t="inlineStr">
         <is>
           <t>75</t>
         </is>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E10" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F10" s="7" t="n">
         <v>6</v>
       </c>
-      <c r="G8" s="9" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="H8" s="10" t="inlineStr">
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="H10" s="10" t="inlineStr">
         <is>
           <t>oui</t>
         </is>
       </c>
-      <c r="I8" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="J8" s="12" t="inlineStr">
+      <c r="I10" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J10" s="12" t="inlineStr">
         <is>
           <t>balises &lt;font&gt; (7) | non responsive</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:J8"/>
+  <autoFilter ref="A3:J10"/>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
@@ -2641,6 +2786,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId7"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>